<commit_message>
Change RAF to 1
</commit_message>
<xml_diff>
--- a/InputData/elec/RAF/Regional Availability Factor.xlsx
+++ b/InputData/elec/RAF/Regional Availability Factor.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\elec\RAF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robbie\Dropbox (Energy Innovation)\My Documents\Energy Policy Solutions\Texas\Models\eps-texas\InputData\elec\RAF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69AC669C-A089-43AC-8C3F-D19C2C3202FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D3CBF88-3903-496A-9A81-DF2D8273E864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23640" activeTab="1" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -245,12 +245,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -720,31 +721,31 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
-        <v>0.6</v>
+      <c r="B2" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>0.9</v>
+      <c r="B3" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4">
-        <v>0.9</v>
+      <c r="B4" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <v>1</v>
       </c>
     </row>
@@ -752,7 +753,7 @@
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <v>1</v>
       </c>
     </row>
@@ -760,7 +761,7 @@
       <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="3">
         <v>1</v>
       </c>
     </row>
@@ -768,7 +769,7 @@
       <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="3">
         <v>1</v>
       </c>
     </row>
@@ -776,7 +777,7 @@
       <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="3">
         <v>1</v>
       </c>
     </row>
@@ -784,7 +785,7 @@
       <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="3">
         <v>1</v>
       </c>
     </row>
@@ -792,120 +793,120 @@
       <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="B11">
-        <v>0.5</v>
+      <c r="B11" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="B12">
-        <v>0.9</v>
+      <c r="B12" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B13">
-        <v>0.9</v>
+      <c r="B13" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B14">
-        <v>0.6</v>
+      <c r="B14" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="B15">
-        <v>0.9</v>
+      <c r="B15" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
-      <c r="B16">
-        <v>0.9</v>
+      <c r="B16" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
-      <c r="B17">
-        <v>0.9</v>
+      <c r="B17" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
-      <c r="B18">
-        <v>0.9</v>
+      <c r="B18" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
-      <c r="B19">
-        <v>0.9</v>
+      <c r="B19" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
-      <c r="B20">
-        <v>0.9</v>
+      <c r="B20" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
-      <c r="B21">
-        <v>0.9</v>
+      <c r="B21" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
-      <c r="B22">
-        <v>0.9</v>
+      <c r="B22" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
-      <c r="B23">
-        <v>0.9</v>
+      <c r="B23" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>50</v>
       </c>
-      <c r="B24">
-        <v>0.9</v>
+      <c r="B24" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>51</v>
       </c>
-      <c r="B25">
-        <v>0.9</v>
+      <c r="B25" s="3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>